<commit_message>
zkb 12519  12520  12521
</commit_message>
<xml_diff>
--- a/src/src/main/webapp/portal/zkb/contract/excel/APM_ZKB_Contract_Exp_Template.xlsx
+++ b/src/src/main/webapp/portal/zkb/contract/excel/APM_ZKB_Contract_Exp_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Intellij Idea\codes\hc-apm-web\src\src\main\webapp\portal\zkb\contract\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBABF639-1D06-4005-AB41-CA91138E1C1D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A38B11-4455-4E9E-BAE8-305E80C0979A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{DFA98752-8825-45D1-95EF-55416474EBE9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{DFA98752-8825-45D1-95EF-55416474EBE9}"/>
   </bookViews>
   <sheets>
     <sheet name="合同" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="相关设备" sheetId="3" r:id="rId3"/>
     <sheet name="相关高值探头" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
   <si>
     <t>代理商</t>
   </si>
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>状态</t>
+  </si>
+  <si>
+    <t>名额扣除类型</t>
   </si>
 </sst>
 </file>
@@ -565,30 +568,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C52200B-3B0C-4F93-BC6C-7CAE122E49C2}">
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.28515625" customWidth="1"/>
-    <col min="13" max="13" width="16.7109375" customWidth="1"/>
-    <col min="14" max="18" width="19.140625" customWidth="1"/>
-    <col min="19" max="19" width="21.42578125" customWidth="1"/>
-    <col min="20" max="23" width="19.140625" customWidth="1"/>
-    <col min="24" max="24" width="16.7109375" customWidth="1"/>
-    <col min="25" max="26" width="19.42578125" customWidth="1"/>
-    <col min="27" max="27" width="21.28515625" customWidth="1"/>
-    <col min="28" max="28" width="23.28515625" customWidth="1"/>
-    <col min="29" max="30" width="26.5703125" customWidth="1"/>
-    <col min="31" max="31" width="29.140625" customWidth="1"/>
-    <col min="32" max="32" width="27.85546875" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" customWidth="1"/>
+    <col min="10" max="10" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" customWidth="1"/>
+    <col min="14" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="19" width="19.140625" customWidth="1"/>
+    <col min="20" max="20" width="21.42578125" customWidth="1"/>
+    <col min="21" max="24" width="19.140625" customWidth="1"/>
+    <col min="25" max="25" width="16.7109375" customWidth="1"/>
+    <col min="26" max="27" width="19.42578125" customWidth="1"/>
+    <col min="28" max="28" width="21.28515625" customWidth="1"/>
+    <col min="29" max="29" width="23.28515625" customWidth="1"/>
+    <col min="30" max="31" width="26.5703125" customWidth="1"/>
+    <col min="32" max="32" width="29.140625" customWidth="1"/>
+    <col min="33" max="33" width="27.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>9</v>
       </c>
@@ -611,78 +615,81 @@
         <v>4</v>
       </c>
       <c r="H1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>